<commit_message>
Update all six prefectures with official Aomori and Fukushima results
</commit_message>
<xml_diff>
--- a/client/public/comparison.xlsx
+++ b/client/public/comparison.xlsx
@@ -14,13 +14,13 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'参考タイム順'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'参考タイム順'!$A$1:$I$16</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'参考タイム順'!$A$1:$I$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'県別1〜4位'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'県別1〜4位'!$A$1:$H$29</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'追加枠・未確認'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'追加枠・未確認'!$A$1:$G$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'追加枠・未確認'!$A$1:$G$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'出典と考察'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'出典と考察'!$A$1:$C$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'出典と考察'!$A$1:$C$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -265,8 +265,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ContenderTimes" displayName="ContenderTimes" ref="A5:I16" headerRowCount="1">
-  <autoFilter ref="A5:I16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ContenderTimes" displayName="ContenderTimes" ref="A5:I20" headerRowCount="1">
+  <autoFilter ref="A5:I20"/>
   <tableColumns count="9">
     <tableColumn id="1" name="参考順"/>
     <tableColumn id="2" name="県"/>
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ExceptionsAndPending" displayName="ExceptionsAndPending" ref="A5:G12" headerRowCount="1">
-  <autoFilter ref="A5:G12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ExceptionsAndPending" displayName="ExceptionsAndPending" ref="A5:G13" headerRowCount="1">
+  <autoFilter ref="A5:G13"/>
   <tableColumns count="7">
     <tableColumn id="1" name="区分"/>
     <tableColumn id="2" name="県"/>
@@ -316,8 +316,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourcesAndNotes" displayName="SourcesAndNotes" ref="A5:C21" headerRowCount="1">
-  <autoFilter ref="A5:C21"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourcesAndNotes" displayName="SourcesAndNotes" ref="A5:C23" headerRowCount="1">
+  <autoFilter ref="A5:C23"/>
   <tableColumns count="3">
     <tableColumn id="1" name="番号・区分"/>
     <tableColumn id="2" name="内容"/>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -647,7 +647,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>確認日：2026年10月24日 17時台（JST）　／　公式結果と補助資料を区別。県間の記録順は予測順位ではありません。</t>
+          <t>確認日：2026年10月31日更新（JST）　／　公式結果と補助資料を区別。県間の記録順は予測順位ではありません。</t>
         </is>
       </c>
     </row>
@@ -926,29 +926,29 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>山形県</t>
+          <t>福島県</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>酒田南</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="n">
-        <v>3</v>
+          <t>ザベリオ</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>2</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>0.05407407407407407</v>
+        <v>0.05347222222222222</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>0.003564814814814815</v>
+        <v>0.002962962962962963</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>0.004513888888888888</v>
+        <v>0.002824074074074074</v>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>公式結果PDF</t>
+          <t>公式結果HTML</t>
         </is>
       </c>
       <c r="I12" s="9" t="inlineStr">
@@ -963,29 +963,29 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>山形県</t>
+          <t>福島県</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>東海大学山形</t>
+          <t>いわき秀英</t>
         </is>
       </c>
       <c r="D13" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E13" s="12" t="n">
-        <v>0.05512731481481482</v>
+        <v>0.05384259259259259</v>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.004618055555555556</v>
+        <v>0.003333333333333334</v>
       </c>
       <c r="G13" s="13" t="n">
-        <v>0.005567129629629629</v>
+        <v>0.003194444444444445</v>
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>公式結果PDF</t>
+          <t>公式結果HTML</t>
         </is>
       </c>
       <c r="I13" s="14" t="inlineStr">
@@ -1000,29 +1000,29 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>岩手県</t>
+          <t>山形県</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>盛岡第三</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="n">
-        <v>2</v>
+          <t>酒田南</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>3</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>0.05650462962962963</v>
+        <v>0.05407407407407407</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>0.005995370370370371</v>
+        <v>0.003564814814814815</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>0.005162037037037037</v>
+        <v>0.004513888888888888</v>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>補助結果・2件照合</t>
+          <t>公式結果PDF</t>
         </is>
       </c>
       <c r="I14" s="9" t="inlineStr">
@@ -1037,29 +1037,29 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>岩手県</t>
+          <t>福島県</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>盛岡大学附属</t>
+          <t>日大東北</t>
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>0.05851851851851852</v>
+        <v>0.05414351851851852</v>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.008009259259259259</v>
+        <v>0.003634259259259259</v>
       </c>
       <c r="G15" s="13" t="n">
-        <v>0.007175925925925926</v>
+        <v>0.00349537037037037</v>
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>補助結果・2件照合</t>
+          <t>公式結果HTML</t>
         </is>
       </c>
       <c r="I15" s="14" t="inlineStr">
@@ -1074,32 +1074,180 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>岩手県</t>
+          <t>山形県</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>盛岡市立</t>
+          <t>東海大学山形</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
         <v>4</v>
       </c>
       <c r="E16" s="7" t="n">
+        <v>0.05512731481481482</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>0.004618055555555556</v>
+      </c>
+      <c r="G16" s="8" t="n">
+        <v>0.005567129629629629</v>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>公式結果PDF</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>出典を開く</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>岩手県</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>盛岡第三</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="12" t="n">
+        <v>0.05650462962962963</v>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>0.005995370370370371</v>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>0.005162037037037037</v>
+      </c>
+      <c r="H17" s="11" t="inlineStr">
+        <is>
+          <t>補助結果・2件照合</t>
+        </is>
+      </c>
+      <c r="I17" s="14" t="inlineStr">
+        <is>
+          <t>出典を開く</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>青森県</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>八戸学院光星</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>0.05688657407407408</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>0.006377314814814815</v>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>0.008738425925925926</v>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>公式結果PDF</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>出典を開く</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>岩手県</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>盛岡大学附属</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <v>0.05851851851851852</v>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>0.008009259259259259</v>
+      </c>
+      <c r="G19" s="13" t="n">
+        <v>0.007175925925925926</v>
+      </c>
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t>補助結果・2件照合</t>
+        </is>
+      </c>
+      <c r="I19" s="14" t="inlineStr">
+        <is>
+          <t>出典を開く</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>岩手県</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>盛岡市立</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" s="7" t="n">
         <v>0.05876157407407408</v>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="F20" s="8" t="n">
         <v>0.008252314814814815</v>
       </c>
-      <c r="G16" s="8" t="n">
+      <c r="G20" s="8" t="n">
         <v>0.007418981481481481</v>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>補助結果・2件照合</t>
         </is>
       </c>
-      <c r="I16" s="9" t="inlineStr">
+      <c r="I20" s="9" t="inlineStr">
         <is>
           <t>出典を開く</t>
         </is>
@@ -1123,12 +1271,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId15"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1169,7 +1321,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>確認日：2026年10月24日 17時台（JST）　／　公式結果と補助資料を区別。県間の記録順は予測順位ではありません。</t>
+          <t>確認日：2026年10月31日更新（JST）　／　公式結果と補助資料を区別。県間の記録順は予測順位ではありません。</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1367,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>青森県</t>
@@ -1226,18 +1378,20 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>未開催・未確定</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="n"/>
+          <t>青森山田</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>0.04814814814814815</v>
+      </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>結果確定待ち</t>
+          <t>対象外・県1位</t>
         </is>
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>公式日程・要項</t>
+          <t>公式結果PDF</t>
         </is>
       </c>
       <c r="G6" s="16" t="inlineStr">
@@ -1247,11 +1401,11 @@
       </c>
       <c r="H6" s="16" t="inlineStr">
         <is>
-          <t>2026-10-29開催予定</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1">
+          <t>公式順位1位。公式PDFで大会新記録と表記。第38回全国・第37回東北高校女子駅伝県予選会の記録表。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>青森県</t>
@@ -1262,18 +1416,20 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>未開催・未確定</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="n"/>
+          <t>八戸学院光星</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>0.05688657407407408</v>
+      </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>結果確定待ち</t>
+          <t>2〜4位対象</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>公式日程・要項</t>
+          <t>公式結果PDF</t>
         </is>
       </c>
       <c r="G7" s="14" t="inlineStr">
@@ -1283,11 +1439,11 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>2026-10-29開催予定</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1">
+          <t>公式順位2位。東北大会実施要項の『女子は各県上位4チーム』に照らし、青森の正式順位校として出場対象。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="64" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>青森県</t>
@@ -1298,18 +1454,18 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>未開催・未確定</t>
+          <t>該当なし（正式順位なし）</t>
         </is>
       </c>
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>結果確定待ち</t>
+          <t>対象校なし</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>公式日程・要項</t>
+          <t>公式結果PDF</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -1319,11 +1475,11 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>2026-10-29開催予定</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="32" customHeight="1">
+          <t>正式順位は青森山田・八戸学院光星の2校のみ。青森山田Ｂ（01:14:37）と大湊・田名部（01:26:17）は公式OP・順位なしで、正式3位・4位は存在しません。OPを3位・4位として補完しません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="64" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>青森県</t>
@@ -1334,18 +1490,18 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>未開催・未確定</t>
+          <t>該当なし（正式順位なし）</t>
         </is>
       </c>
       <c r="D9" s="11" t="n"/>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>結果確定待ち</t>
+          <t>対象校なし</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>公式日程・要項</t>
+          <t>公式結果PDF</t>
         </is>
       </c>
       <c r="G9" s="14" t="inlineStr">
@@ -1355,7 +1511,7 @@
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>2026-10-29開催予定</t>
+          <t>正式順位は青森山田・八戸学院光星の2校のみ。青森山田Ｂ（01:14:37）と大湊・田名部（01:26:17）は公式OP・順位なしで、正式3位・4位は存在しません。OPを3位・4位として補完しません。</t>
         </is>
       </c>
     </row>
@@ -1969,7 +2125,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="32" customHeight="1">
+    <row r="26" ht="36" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
           <t>福島県</t>
@@ -1980,18 +2136,20 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>未開催・未確定</t>
-        </is>
-      </c>
-      <c r="D26" s="16" t="n"/>
+          <t>学法石川</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="n">
+        <v>0.05064814814814815</v>
+      </c>
       <c r="E26" s="16" t="inlineStr">
         <is>
-          <t>結果確定待ち</t>
+          <t>対象外・県1位</t>
         </is>
       </c>
       <c r="F26" s="16" t="inlineStr">
         <is>
-          <t>公式日程・要項</t>
+          <t>公式結果HTML</t>
         </is>
       </c>
       <c r="G26" s="16" t="inlineStr">
@@ -2001,11 +2159,11 @@
       </c>
       <c r="H26" s="16" t="inlineStr">
         <is>
-          <t>2026-10-31開催予定</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="32" customHeight="1">
+          <t>福島陸協公式の女子総合成績による正式1位。東北大会出場（TUF当日報道は女子上位4チームの出場を明記）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="50" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>福島県</t>
@@ -2016,18 +2174,20 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>未開催・未確定</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="n"/>
+          <t>ザベリオ</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="n">
+        <v>0.05347222222222222</v>
+      </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>結果確定待ち</t>
+          <t>2〜4位対象</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>公式日程・要項</t>
+          <t>公式結果HTML</t>
         </is>
       </c>
       <c r="G27" s="14" t="inlineStr">
@@ -2037,7 +2197,7 @@
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>2026-10-31開催予定</t>
+          <t>福島陸協公式の女子総合成績による正式2位。東北大会出場。TUF記事中の「ザベリオ学園」ではなく、県公式結果のチーム表記を採用。</t>
         </is>
       </c>
     </row>
@@ -2052,18 +2212,20 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>未開催・未確定</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="n"/>
+          <t>いわき秀英</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>0.05384259259259259</v>
+      </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>結果確定待ち</t>
+          <t>2〜4位対象</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>公式日程・要項</t>
+          <t>公式結果HTML</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
@@ -2073,7 +2235,7 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>2026-10-31開催予定</t>
+          <t>福島陸協公式の女子総合成績による正式3位。東北大会出場。</t>
         </is>
       </c>
     </row>
@@ -2088,18 +2250,20 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>未開催・未確定</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="n"/>
+          <t>日大東北</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="n">
+        <v>0.05414351851851852</v>
+      </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>結果確定待ち</t>
+          <t>2〜4位対象</t>
         </is>
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>公式日程・要項</t>
+          <t>公式結果HTML</t>
         </is>
       </c>
       <c r="G29" s="14" t="inlineStr">
@@ -2109,7 +2273,7 @@
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>2026-10-31開催予定</t>
+          <t>福島陸協公式の女子総合成績による正式4位。東北大会出場。</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2189,7 +2353,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>確認日：2026年10月24日 17時台（JST）　／　公式結果と補助資料を区別。県間の記録順は予測順位ではありません。</t>
+          <t>確認日：2026年10月31日更新（JST）　／　公式結果と補助資料を区別。県間の記録順は予測順位ではありません。</t>
         </is>
       </c>
     </row>
@@ -2389,10 +2553,10 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="48" customHeight="1">
+    <row r="11" ht="50" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>未開催</t>
+          <t>正式順位なし</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
@@ -2402,14 +2566,14 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>2〜4位は未確定</t>
+          <t>3位・4位の対象校なし</t>
         </is>
       </c>
       <c r="D11" s="11" t="n"/>
       <c r="E11" s="11" t="n"/>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>2026-10-29開催予定。過年度の記録は代用しない。</t>
+          <t>正式順位は青森山田・八戸学院光星の2校のみ。青森山田Ｂ（01:14:37）と大湊・田名部（01:26:17）は公式OP・順位なしで、正式3位・4位は存在しません。OPを3位・4位として補完しません。</t>
         </is>
       </c>
       <c r="G11" s="14" t="inlineStr">
@@ -2421,27 +2585,60 @@
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>未開催</t>
+          <t>県予選OP</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>福島県</t>
+          <t>青森県</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>2〜4位は未確定</t>
+          <t>青森山田Ｂ</t>
         </is>
       </c>
       <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
+      <c r="E12" s="7" t="n">
+        <v>0.05181712962962963</v>
+      </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>2026-10-31開催予定。過年度の記録は代用しない。</t>
+          <t>県予選OP・正式順位なし。県2〜4位の参考順に含めない。</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>出典を開く</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>県予選OP</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>青森県</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>大湊・田名部</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="12" t="n">
+        <v>0.05991898148148148</v>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>県予選OP・正式順位なし。県2〜4位の参考順に含めない。</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
         <is>
           <t>出典を開く</t>
         </is>
@@ -2461,12 +2658,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId8"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2477,7 +2675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2502,7 +2700,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>確認日：2026年10月24日 17時台（JST）　／　公式結果と補助資料を区別。県間の記録順は予測順位ではありません。</t>
+          <t>確認日：2026年10月31日更新（JST）　／　公式結果と補助資料を区別。県間の記録順は予測順位ではありません。</t>
         </is>
       </c>
     </row>
@@ -2616,7 +2814,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>岩手県 2026年女子県高校駅伝の結果資料</t>
+          <t>福島県 2026年女子県高校駅伝の結果資料</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -2633,7 +2831,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>青森県 2026年女子県高校駅伝の公式日程・要項</t>
+          <t>岩手県 2026年女子県高校駅伝の結果資料</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -2650,7 +2848,7 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>福島県 2026年女子県高校駅伝の公式日程・要項</t>
+          <t>青森県 2026年女子県高校駅伝の結果資料</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
@@ -2714,7 +2912,7 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>県3・4位校の中で最も速い確認記録は宮城県の聖和学園で、1時間15分23秒です。全体参考3番目に入るため、県2位だけの比較では対象校の見え方が変わります。</t>
+          <t>今回追加した青森県の2位は八戸学院光星で、1時間21分55秒、全体の参考順は13番目です。先頭の確認記録との差は551秒です。県代表の1位校はこの比較から除いています。</t>
         </is>
       </c>
       <c r="C17" s="11" t="n"/>
@@ -2727,7 +2925,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>秋田北鷹と秋田工業の差は15秒です。県3位の秋田工業も含め、当日のオーダーや区間ごとの走りで逆転し得る候補として見るのが適切です。</t>
+          <t>今回追加した福島県の2位はザベリオで、1時間17分00秒、全体の参考順は7番目です。先頭の確認記録との差は256秒です。県代表の1位校はこの比較から除いています。</t>
         </is>
       </c>
       <c r="C18" s="6" t="n"/>
@@ -2740,7 +2938,7 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>宮城4位の古川学園と秋田2位の秋田北鷹の記録差は1秒です。県内順位が違っても総合記録は近く、県4位校を除くと比較から漏れる例です。</t>
+          <t>県3・4位校の中で最も速い確認記録は宮城県の聖和学園で、1時間15分23秒です。全体参考3番目に入るため、県2位だけの比較では対象校の見え方が変わります。</t>
         </is>
       </c>
       <c r="C19" s="11" t="n"/>
@@ -2753,7 +2951,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>山形県予選と東北大会は同じ長井市の会場名・周回コースで案内されていますが、区間設定や当日の条件を同一と決めつけることはできません。県間の総合タイムから勝率を算出したり、出場権の獲得を断定したりはしていません。</t>
+          <t>秋田北鷹と秋田工業の差は15秒です。県3位の秋田工業も含め、当日のオーダーや区間ごとの走りで逆転し得る候補として見るのが適切です。</t>
         </is>
       </c>
       <c r="C20" s="6" t="n"/>
@@ -2766,10 +2964,36 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>青森・福島の予選が終わるまでは全県の比較が完成していません。比較対象の県2〜4位校も、正式な東北大会出場名簿と実際の県代表校を確認してから全国地区代表の候補を確定します。</t>
+          <t>宮城4位の古川学園と秋田2位の秋田北鷹の記録差は1秒です。県内順位が違っても総合記録は近く、県4位校を除くと比較から漏れる例です。</t>
         </is>
       </c>
       <c r="C21" s="11" t="n"/>
+    </row>
+    <row r="22" ht="54" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>考察</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>山形県予選と東北大会は同じ長井市の会場名・周回コースで案内されていますが、区間設定や当日の条件を同一と決めつけることはできません。県間の総合タイムから勝率を算出したり、出場権の獲得を断定したりはしていません。</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n"/>
+    </row>
+    <row r="23" ht="54" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>考察</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>青森・福島を加え、全6県の予選結果を反映しました。県2〜4位の記録確認済み15校を比較し、タイム未確認1校は参考順から除外しています。出場権を争う最終対象校は、東北大会の正式出場名簿と実際の県代表校で確認してください。</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>